<commit_message>
#172 J1 header FOB P3 Header TDS Updated in BOM
</commit_message>
<xml_diff>
--- a/BOM/Fob_Transmitter/JLCPCB-BOM.xlsx
+++ b/BOM/Fob_Transmitter/JLCPCB-BOM.xlsx
@@ -126,9 +126,6 @@
     <t>C14664</t>
   </si>
   <si>
-    <t>C2718488</t>
-  </si>
-  <si>
     <t>C492404</t>
   </si>
   <si>
@@ -160,6 +157,9 @@
   </si>
   <si>
     <t>C381208</t>
+  </si>
+  <si>
+    <t>C358717</t>
   </si>
 </sst>
 </file>
@@ -328,7 +328,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -359,6 +359,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -667,7 +670,7 @@
         <v>23</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -722,8 +725,8 @@
       <c r="C5" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="D5" s="6" t="s">
-        <v>35</v>
+      <c r="D5" s="11" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -737,7 +740,7 @@
         <v>26</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -751,7 +754,7 @@
         <v>27</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -765,7 +768,7 @@
         <v>28</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -779,7 +782,7 @@
         <v>29</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -793,7 +796,7 @@
         <v>8</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -807,7 +810,7 @@
         <v>30</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -821,21 +824,21 @@
         <v>31</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B13" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="C13" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13" s="9" t="s">
         <v>45</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="D13" s="9" t="s">
-        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>